<commit_message>
Add claims and notices skills; fix Excel Setup references
claims: progress claim and ex GST computations, a progress payments page,
and invoice and calculator examples. notices: delay notification, site
instruction and back charge, with an add_days date computation and a
site instructions and back charges page.

fill_template.py gains add_row, delete_row and tick for Word templates
and input-cell filling for Excel, and reads project and spec values as
typed. Fixes off-by-one Setup sheet references in 21 workbooks, which
showed blank project names, the contract number as the contract sum and
retention calculated from the contract sum; okf_lint.py now checks them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/excel/Allowances_Register_TEMPLATE.xlsx
+++ b/templates/excel/Allowances_Register_TEMPLATE.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Instructions" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -740,14 +740,14 @@
         <v>17</v>
       </c>
       <c r="B2" s="5" t="n">
-        <f aca="false">Setup!B12</f>
+        <f aca="false">Setup!B13</f>
         <v>0</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="F2" s="5" t="n">
-        <f aca="false">Setup!B14</f>
+        <f aca="false">Setup!B15</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>